<commit_message>
Revisión en Excel: script 12 pasa LISTA_REVISION_TA.xlsx a TA.xlsx (opción «De acuerdo»)
- 12_aplicar_lista_revision.py: valida y aplica MI DECISIÓN/CRITERIO/COMENTARIO; modo --probar
- 09: la confianza de la IA solo aparece en filas aún no verificadas
- LISTA_REVISION_TA.xlsx: lista desplegable con «De acuerdo» e instrucciones de llenado

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BxN9W1XmdV2QxsHjBBQujW
</commit_message>
<xml_diff>
--- a/RSL/cribado/revision/LISTA_REVISION_TA.xlsx
+++ b/RSL/cribado/revision/LISTA_REVISION_TA.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -460,9 +460,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -491,9 +489,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr"/>
-    </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
@@ -508,9 +504,7 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr"/>
-    </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
@@ -522,6 +516,58 @@
       <c r="A12" t="inlineStr">
         <is>
           <t>Criterios y prompt para ayudarte: ver cribado/GUIA_REVISION_TA.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CÓMO LLENAR (para que el script 12 lo pase a TA.xlsx y a Parsif.al):</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  MI DECISIÓN = «De acuerdo»  → se acepta la propuesta tal cual (decisión, criterio y motivo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  MI DECISIÓN = Incluir / Duda → cambia a esa decisión; MI CRITERIO vacío.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  MI DECISIÓN = Excluir → MI CRITERIO obligatorio (CE-1, CE-2, CE-3, CE-4, CE-5, CI-2 o CI-3).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  MI COMENTARIO = tu motivo en una frase. Si lo dejas vacío, se usa el motivo de la IA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Filas sin MI DECISIÓN = no revisadas: se quedan como estaban.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Después: python cribado\scripts\12_aplicar_lista_revision.py   y luego   python cribado\scripts\09_generar_script_parsifal.py</t>
         </is>
       </c>
     </row>
@@ -10290,10 +10336,10 @@
   </sheetData>
   <autoFilter ref="A1:P152"/>
   <dataValidations count="2">
-    <dataValidation sqref="N2:N152" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Incluir,Duda,Excluir"</formula1>
+    <dataValidation sqref="N2:N152" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"De acuerdo,Incluir,Duda,Excluir"</formula1>
     </dataValidation>
-    <dataValidation sqref="O2:O152" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="O2:O152" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"CE-1,CE-2,CE-3,CE-4,CE-5,CI-2,CI-3"</formula1>
     </dataValidation>
   </dataValidations>
@@ -14736,10 +14782,10 @@
   </sheetData>
   <autoFilter ref="A1:P58"/>
   <dataValidations count="2">
-    <dataValidation sqref="N2:N58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Incluir,Duda,Excluir"</formula1>
+    <dataValidation sqref="N2:N58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"De acuerdo,Incluir,Duda,Excluir"</formula1>
     </dataValidation>
-    <dataValidation sqref="O2:O58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="O2:O58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"CE-1,CE-2,CE-3,CE-4,CE-5,CI-2,CI-3"</formula1>
     </dataValidation>
   </dataValidations>
@@ -44251,10 +44297,10 @@
   </sheetData>
   <autoFilter ref="A1:P456"/>
   <dataValidations count="2">
-    <dataValidation sqref="N2:N456" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Incluir,Duda,Excluir"</formula1>
+    <dataValidation sqref="N2:N456" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"De acuerdo,Incluir,Duda,Excluir"</formula1>
     </dataValidation>
-    <dataValidation sqref="O2:O456" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="O2:O456" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"CE-1,CE-2,CE-3,CE-4,CE-5,CI-2,CI-3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>